<commit_message>
data: actualizar BD REM, Inflacion mensual y Letras Activas
- BD REM.xlsx: nuevas proyecciones REM BCRA
- Inflacion mensual.xlsx: IPC INDEC actualizado
- Letras Activas.xlsx: letras y boncaps vigentes

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/BD REM.xlsx
+++ b/backend/data/BD REM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1ftoIZqhxjIK-zxyM2xIG9xFIX4GG9BvJ\DCF\Marketing\Instagram\Scripts Python\App DCF Dani\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1ftoIZqhxjIK-zxyM2xIG9xFIX4GG9BvJ\DCF\Claude\dcf-herramientas-web\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDA1340F-69C2-4647-9E22-3DE604E63EAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC692F7B-FA0F-45F7-A090-CC3220E605D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CB73FF54-44C1-4E27-A365-D53B7B4CE952}"/>
   </bookViews>
@@ -48,10 +48,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -147,7 +146,7 @@
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="167" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -157,10 +156,10 @@
     <xf numFmtId="10" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="4" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -542,7 +541,7 @@
         <v>46113</v>
       </c>
       <c r="B5" s="6">
-        <v>2.5705335165110199</v>
+        <v>2.635915686224175</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
@@ -550,7 +549,7 @@
         <v>46143</v>
       </c>
       <c r="B6" s="5">
-        <v>2.2317104245191031</v>
+        <v>2.2867443141716119</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.35">
@@ -558,7 +557,7 @@
         <v>46174</v>
       </c>
       <c r="B7" s="6">
-        <v>2.038777101239948</v>
+        <v>2.0732407212048471</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.35">
@@ -566,7 +565,7 @@
         <v>46204</v>
       </c>
       <c r="B8" s="5">
-        <v>1.9688550797838209</v>
+        <v>2.054743329977732</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
@@ -574,22 +573,24 @@
         <v>46235</v>
       </c>
       <c r="B9" s="6">
-        <v>1.8004639144284269</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+        <v>1.8950276844426019</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>46266</v>
       </c>
       <c r="B10" s="5">
-        <v>1.7589175909647601</v>
+        <v>1.881652139799723</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="1">
         <v>46296</v>
       </c>
-      <c r="B11" s="4"/>
+      <c r="B11" s="5">
+        <v>1.8</v>
+      </c>
     </row>
     <row r="12" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1">

</xml_diff>

<commit_message>
Actualizacion Dato Infla Mayo
</commit_message>
<xml_diff>
--- a/backend/data/BD REM.xlsx
+++ b/backend/data/BD REM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\.shortcut-targets-by-id\1ftoIZqhxjIK-zxyM2xIG9xFIX4GG9BvJ\DCF\Claude\dcf-herramientas-web\backend\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC692F7B-FA0F-45F7-A090-CC3220E605D8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{014D54D1-5F7C-4951-A749-0212F21A30D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{CB73FF54-44C1-4E27-A365-D53B7B4CE952}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CB73FF54-44C1-4E27-A365-D53B7B4CE952}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>Mes</t>
   </si>
   <si>
     <t>REM</t>
+  </si>
+  <si>
+    <t>1.8</t>
+  </si>
+  <si>
+    <t>1.7</t>
   </si>
 </sst>
 </file>
@@ -532,17 +538,13 @@
       <c r="A4" s="1">
         <v>46082</v>
       </c>
-      <c r="B4" s="5">
-        <v>3</v>
-      </c>
+      <c r="B4" s="5"/>
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>46113</v>
       </c>
-      <c r="B5" s="6">
-        <v>2.635915686224175</v>
-      </c>
+      <c r="B5" s="6"/>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
@@ -565,15 +567,15 @@
         <v>46204</v>
       </c>
       <c r="B8" s="5">
-        <v>2.054743329977732</v>
+        <v>2</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>46235</v>
       </c>
-      <c r="B9" s="6">
-        <v>1.8950276844426019</v>
+      <c r="B9" s="6" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.35">
@@ -584,7 +586,7 @@
         <v>1.881652139799723</v>
       </c>
     </row>
-    <row r="11" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>46296</v>
       </c>
@@ -592,11 +594,13 @@
         <v>1.8</v>
       </c>
     </row>
-    <row r="12" spans="1:2" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>46327</v>
       </c>
-      <c r="B12" s="4"/>
+      <c r="B12" s="5" t="s">
+        <v>3</v>
+      </c>
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.35">
       <c r="A13" s="1">

</xml_diff>